<commit_message>
finished connect database and working on mobile verison
</commit_message>
<xml_diff>
--- a/QuotationData.xlsx
+++ b/QuotationData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sdani\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33FBECF2-5817-4190-A3C5-FC39DF462868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A05B065-0F32-4870-AEF3-EF0ECC987F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,117 +20,141 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="284">
   <si>
     <t>Date</t>
   </si>
   <si>
+    <t>QuotationNo</t>
+  </si>
+  <si>
+    <t>CreatedBy</t>
+  </si>
+  <si>
+    <t>ClientName</t>
+  </si>
+  <si>
+    <t>ContactPerson</t>
+  </si>
+  <si>
+    <t>ContactNo</t>
+  </si>
+  <si>
+    <t>Subtotal</t>
+  </si>
+  <si>
+    <t>VAT</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>ItemsJSON</t>
+  </si>
+  <si>
+    <t>Qudra Company Ltd</t>
+  </si>
+  <si>
+    <t>MME</t>
+  </si>
+  <si>
+    <t>QT-260529001</t>
+  </si>
+  <si>
+    <t>Afro</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NETKOM </t>
+  </si>
+  <si>
+    <t>Irfan Mehmood</t>
+  </si>
+  <si>
+    <t>[{"code":"LT","desc":"Safety Shoes Italian","qty":4,"unitPrice":70},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":4,"unitPrice":13},{"code":"GWH-30","desc":"Ironcap - Working At Height Helmet ","qty":1,"unitPrice":65},{"code":"LT","desc":"Combination Wrench Set (6-32) 25 pcs","qty":1,"unitPrice":115},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":1,"unitPrice":40},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":1,"unitPrice":20},{"code":"LT","desc":"Cutter Plier (Dewesser Germany)","qty":1,"unitPrice":18}]</t>
+  </si>
+  <si>
+    <t>QT-260529002</t>
+  </si>
+  <si>
+    <t>MAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro </t>
+  </si>
+  <si>
+    <t>[{"code":"NM-001","desc":"Engineer Helmet","qty":4,"unitPrice":30},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":4,"unitPrice":13},{"code":"H110","desc":"Brother-H110","qty":2,"unitPrice":180},{"code":"LT","desc":"Multimeter (SANWA)","qty":2,"unitPrice":180},{"code":"LT","desc":"AC/DC Clamp Meter ","qty":2,"unitPrice":170},{"code":"LT","desc":"Powder Fire Extinguisher 3 kg With 6 Months Sticker","qty":2,"unitPrice":50},{"code":"LT","desc":"Warning Tape 200m","qty":1,"unitPrice":15},{"code":"FAK-100","desc":"First Aid Kit","qty":2,"unitPrice":60},{"code":"LT","desc":"Electrical Gloves Class 0 ","qty":3,"unitPrice":65},{"code":"LT","desc":"Safety Shoes Italian","qty":2,"unitPrice":70},{"code":"LT","desc":"Electrical Plier (Dewesser Germany)","qty":2,"unitPrice":18},{"code":"LT","desc":"Long Nose Plier (Dewesser Germany)","qty":2,"unitPrice":18},{"code":"LT","desc":"Steel Tool Box","qty":2,"unitPrice":65},{"code":"LT","desc":"Insulated Screw Driver Set With Tester China","qty":2,"unitPrice":35},{"code":"ISS-100","desc":"Insulated Spanners Set (6-22)","qty":2,"unitPrice":50},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":4,"unitPrice":40},{"code":"LT","desc":"Tie Cutter ","qty":2,"unitPrice":20},{"code":"LT","desc":"Cable Cutter 10\"","qty":2,"unitPrice":25},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":2,"unitPrice":20},{"code":"LT","desc":"Claw Hammer","qty":2,"unitPrice":20},{"code":"LT","desc":"Tester ","qty":2,"unitPrice":7},{"code":"LT","desc":"Zamil Aluminium Ladder 3 Step","qty":3,"unitPrice":125},{"code":"LT","desc":"Adjustable Wrench 12\" Insulated ","qty":2,"unitPrice":40},{"code":"LT","desc":"Measuring Tape 10m (Dewesser Germany)","qty":2,"unitPrice":25},{"code":"LT","desc":"Crimping Tool RJ 45","qty":2,"unitPrice":60},{"code":"LT","desc":"Drill Machine","qty":1,"unitPrice":190},{"code":"LT","desc":"Heat Gun","qty":1,"unitPrice":60},{"code":"LT","desc":"Water Cooler (5 Gallon) ","qty":2,"unitPrice":70},{"code":"LT","desc":"RJ 45 Tester","qty":2,"unitPrice":55},{"code":"LT","desc":"Cable Drum 50M Germany","qty":3,"unitPrice":125},{"code":"LT","desc":"Hand Crimping Tool 6-50mm","qty":2,"unitPrice":85}]</t>
+  </si>
+  <si>
+    <t>QT-260530003</t>
+  </si>
+  <si>
+    <t>Swedtel Company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Irfan Mehmood </t>
+  </si>
+  <si>
+    <t>[{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":7,"unitPrice":13},{"code":"LT","desc":"Water Cooler (5 Gallon) ","qty":2,"unitPrice":70},{"code":"LT","desc":"Safety Shoes Italian","qty":5,"unitPrice":70},{"code":"GWH-30","desc":"Ironcap - Working At Height Helmet ","qty":1,"unitPrice":65},{"code":"HDL-001","desc":"Head lights","qty":2,"unitPrice":25},{"code":"LT","desc":"Cable Cutter 8\" ","qty":2,"unitPrice":22},{"code":"LT","desc":"Cable Cutter 10\"","qty":3,"unitPrice":25},{"code":"LT","desc":"Screw Driver (+) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Screw Driver (-) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Tie Cutter ","qty":5,"unitPrice":20},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":4,"unitPrice":20},{"code":"LT","desc":"Heat Gun","qty":1,"unitPrice":60},{"code":"LT","desc":"Silicon Gun","qty":1,"unitPrice":7},{"code":"LT","desc":"Flood Light 400 Watt","qty":1,"unitPrice":90},{"code":"ISS-100","desc":"Insulated Spanners Set (6-22)","qty":1,"unitPrice":50}]</t>
+  </si>
+  <si>
+    <t>Technical Solution Co</t>
+  </si>
+  <si>
+    <t>BM</t>
+  </si>
+  <si>
+    <t>QT-260531004</t>
+  </si>
+  <si>
+    <t>staff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Vision Contractring Company </t>
+  </si>
+  <si>
+    <t>Rawasy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Irfan </t>
+  </si>
+  <si>
+    <t>[{"code":"GH-60","desc":"Guardian Pro - 5D Harness","qty":1,"unitPrice":400},{"code":"GH-50","desc":"Fortress Pro - 5D Harness","qty":1,"unitPrice":350},{"code":"GDL-230","desc":"Titan Twin Static - Double Lanyard","qty":1,"unitPrice":210},{"code":"GDL-330","desc":"Titan Twin Shock- Double Lanyard","qty":1,"unitPrice":210},{"code":"GP-30","desc":"AnchorLine Adjust - Position Lanyard ","qty":1,"unitPrice":160},{"code":"GP-230","desc":"Ironhold Adjust - Position Lanyard ","qty":1,"unitPrice":160},{"code":"GSL-120","desc":"Anchorcore - Sling","qty":1,"unitPrice":30},{"code":"GCL-W100","desc":"Ironclamp - Wire Cab Lock","qty":1,"unitPrice":160},{"code":"GCL-S200","desc":"Ascendrail - Slide Cab Lock ","qty":1,"unitPrice":1000},{"code":"GSG-13","desc":"GripX - Safety Gloves","qty":1,"unitPrice":3},{"code":"GSG-21","desc":"GripX Pro - Safety Gloves","qty":1,"unitPrice":8},{"code":"ISS-100","desc":"Insulated Spanners Set (6-22)","qty":1,"unitPrice":50},{"code":"GRF-A10","desc":"Guard - Rope Fall Arrestor","qty":1,"unitPrice":300},{"code":"GRF-A20","desc":"Guard - Rope Fall Arrestor","qty":1,"unitPrice":300},{"code":"GR-P200","desc":"Anchorline - Rope 200M","qty":1,"unitPrice":700},{"code":"GWH-30","desc":"Ironcap - Working At Height Helmet ","qty":1,"unitPrice":70},{"code":"NM-001","desc":"Engineer Helmet","qty":1,"unitPrice":30},{"code":"GCR-100","desc":"Corelock - Carabiner","qty":1,"unitPrice":15},{"code":"H110","desc":"Label Machine Brother","qty":1,"unitPrice":180},{"code":"GRB-25","desc":"Rigger Bag","qty":1,"unitPrice":70},{"code":"FAK-100","desc":"First Aid Kit","qty":1,"unitPrice":65},{"code":"LT","desc":"Bosch Laser Meter 150m","qty":1,"unitPrice":1400},{"code":"LT","desc":"Multimeter (SANWA)","qty":1,"unitPrice":180},{"code":"LT","desc":"AC/DC Clamp Meter ","qty":1,"unitPrice":170},{"code":"LT","desc":"Clamp Meter (Kuoritsu)","qty":1,"unitPrice":190},{"code":"LT","desc":"Crimping Tool RJ 45","qty":1,"unitPrice":60},{"code":"LT","desc":"Power Crimper 6-50MM Size","qty":1,"unitPrice":85},{"code":"LT","desc":"RJ 45 Tester","qty":1,"unitPrice":55},{"code":"LT","desc":"Combination Wrench Set (6-32) 14 pcs Insulated","qty":1,"unitPrice":65},{"code":"LT","desc":"Combination Wrench Set (6-32) 25 pcs Insulated","qty":1,"unitPrice":115},{"code":"CMP-001","desc":"Compass","qty":1,"unitPrice":100},{"code":"CMPD-001","desc":"Digital Compass","qty":1,"unitPrice":200},{"code":"LT","desc":"Compass With Mirror ","qty":1,"unitPrice":75},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":1,"unitPrice":20},{"code":"LT","desc":"Socket Wrench Set 24 pcs 1/2\"","qty":1,"unitPrice":125},{"code":"LT","desc":"Adjustable Wrench 10\"","qty":1,"unitPrice":30},{"code":"LT","desc":"Adjustable Wrench 12\"","qty":1,"unitPrice":40},{"code":"LT","desc":"Screw Driver (+) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Screw Driver (-) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Insulated Screw Driver Set With Tester","qty":1,"unitPrice":70},{"code":"LT","desc":"Insulated Screw Driver Set With Tester China","qty":1,"unitPrice":35},{"code":"LT","desc":"Hacksaw Frame With Blade","qty":1,"unitPrice":18},{"code":"LT","desc":"Allen Key Set 1.5–10mm","qty":1,"unitPrice":60},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":1,"unitPrice":40},{"code":"LT","desc":"Electrical Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Long Nose Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Cutter Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Vice Grip Plier 10\"","qty":1,"unitPrice":35},{"code":"LT","desc":"Cable Cutter 8\" ","qty":1,"unitPrice":22},{"code":"LT","desc":"Cable Cutter 10\"","qty":1,"unitPrice":25},{"code":"LT","desc":"Tie Cutter ","qty":1,"unitPrice":20},{"code":"LT","desc":"Safety Shoes Italian","qty":1,"unitPrice":70},{"code":"LT","desc":"Electrical Gloves Class 1","qty":1,"unitPrice":85},{"code":"LT","desc":"Electrical Gloves Class 0 ","qty":1,"unitPrice":65},{"code":"LT","desc":"Zamil Aluminium Ladder 3 Step","qty":1,"unitPrice":125},{"code":"LT","desc":"Zamil Aluminium Ladder 5 Step","qty":1,"unitPrice":180},{"code":"LT","desc":"Flood Light 400 Watt","qty":1,"unitPrice":90},{"code":"LT","desc":"Heat Gun","qty":1,"unitPrice":60},{"code":"LT","desc":"Drill Machine","qty":1,"unitPrice":190},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":1,"unitPrice":13},{"code":"GBV-100-XL","desc":"ViziGuard - Safety Vest","qty":1,"unitPrice":13},{"code":"LT","desc":"Measuring Tape 10m (Dewesser Germany)","qty":1,"unitPrice":25},{"code":"HDL-001","desc":"Head lights","qty":1,"unitPrice":25},{"code":"LT","desc":"3M Eye Protection Googles ","qty":1,"unitPrice":40},{"code":"GRK-100","desc":"ResQ Pro - Rescue Kit ","qty":1,"unitPrice":1300},{"code":"LT","desc":"Measuring Tape 5m (Dewesser Germany)","qty":1,"unitPrice":15},{"code":"LT","desc":"Measuring Tape 30M","qty":1,"unitPrice":35},{"code":"LT","desc":"Measuring Tape 50M","qty":1,"unitPrice":45}]</t>
+  </si>
+  <si>
+    <t>Dorr-Almas.Est</t>
+  </si>
+  <si>
+    <t>DAEM COMPANY FOR TRADING</t>
+  </si>
+  <si>
+    <t>I-man co</t>
+  </si>
+  <si>
+    <t>Xad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company KAREEM SWAR </t>
+  </si>
+  <si>
+    <t>QT-260531005</t>
+  </si>
+  <si>
+    <t>Smart lines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adil Awan </t>
+  </si>
+  <si>
+    <t>Alpha Global</t>
+  </si>
+  <si>
     <t>GTEL</t>
   </si>
   <si>
-    <t>QuotationNo</t>
-  </si>
-  <si>
-    <t>CreatedBy</t>
-  </si>
-  <si>
-    <t>ClientName</t>
-  </si>
-  <si>
-    <t>ContactPerson</t>
-  </si>
-  <si>
-    <t>ContactNo</t>
-  </si>
-  <si>
-    <t>Subtotal</t>
-  </si>
-  <si>
-    <t>VAT</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>ItemsJSON</t>
-  </si>
-  <si>
-    <t>QT-260529001</t>
-  </si>
-  <si>
-    <t>admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NETKOM </t>
-  </si>
-  <si>
-    <t>Irfan Mehmood</t>
-  </si>
-  <si>
-    <t>Qudra Company Ltd</t>
-  </si>
-  <si>
-    <t>MME</t>
-  </si>
-  <si>
-    <t>Afro</t>
-  </si>
-  <si>
-    <t>[{"code":"LT","desc":"Safety Shoes Italian","qty":4,"unitPrice":70},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":4,"unitPrice":13},{"code":"GWH-30","desc":"Ironcap - Working At Height Helmet ","qty":1,"unitPrice":65},{"code":"LT","desc":"Combination Wrench Set (6-32) 25 pcs","qty":1,"unitPrice":115},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":1,"unitPrice":40},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":1,"unitPrice":20},{"code":"LT","desc":"Cutter Plier (Dewesser Germany)","qty":1,"unitPrice":18}]</t>
-  </si>
-  <si>
-    <t>QT-260529002</t>
-  </si>
-  <si>
-    <t>MAS</t>
-  </si>
-  <si>
-    <t>[{"code":"NM-001","desc":"Engineer Helmet","qty":4,"unitPrice":30},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":4,"unitPrice":13},{"code":"H110","desc":"Brother-H110","qty":2,"unitPrice":180},{"code":"LT","desc":"Multimeter (SANWA)","qty":2,"unitPrice":180},{"code":"LT","desc":"AC/DC Clamp Meter ","qty":2,"unitPrice":170},{"code":"LT","desc":"Powder Fire Extinguisher 3 kg With 6 Months Sticker","qty":2,"unitPrice":50},{"code":"LT","desc":"Warning Tape 200m","qty":1,"unitPrice":15},{"code":"FAK-100","desc":"First Aid Kit","qty":2,"unitPrice":60},{"code":"LT","desc":"Electrical Gloves Class 0 ","qty":3,"unitPrice":65},{"code":"LT","desc":"Safety Shoes Italian","qty":2,"unitPrice":70},{"code":"LT","desc":"Electrical Plier (Dewesser Germany)","qty":2,"unitPrice":18},{"code":"LT","desc":"Long Nose Plier (Dewesser Germany)","qty":2,"unitPrice":18},{"code":"LT","desc":"Steel Tool Box","qty":2,"unitPrice":65},{"code":"LT","desc":"Insulated Screw Driver Set With Tester China","qty":2,"unitPrice":35},{"code":"ISS-100","desc":"Insulated Spanners Set (6-22)","qty":2,"unitPrice":50},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":4,"unitPrice":40},{"code":"LT","desc":"Tie Cutter ","qty":2,"unitPrice":20},{"code":"LT","desc":"Cable Cutter 10\"","qty":2,"unitPrice":25},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":2,"unitPrice":20},{"code":"LT","desc":"Claw Hammer","qty":2,"unitPrice":20},{"code":"LT","desc":"Tester ","qty":2,"unitPrice":7},{"code":"LT","desc":"Zamil Aluminium Ladder 3 Step","qty":3,"unitPrice":125},{"code":"LT","desc":"Adjustable Wrench 12\" Insulated ","qty":2,"unitPrice":40},{"code":"LT","desc":"Measuring Tape 10m (Dewesser Germany)","qty":2,"unitPrice":25},{"code":"LT","desc":"Crimping Tool RJ 45","qty":2,"unitPrice":60},{"code":"LT","desc":"Drill Machine","qty":1,"unitPrice":190},{"code":"LT","desc":"Heat Gun","qty":1,"unitPrice":60},{"code":"LT","desc":"Water Cooler (5 Gallon) ","qty":2,"unitPrice":70},{"code":"LT","desc":"RJ 45 Tester","qty":2,"unitPrice":55},{"code":"LT","desc":"Cable Drum 50M Germany","qty":3,"unitPrice":125},{"code":"LT","desc":"Hand Crimping Tool 6-50mm","qty":2,"unitPrice":85}]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metro </t>
-  </si>
-  <si>
-    <t>QT-260530003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Irfan Mehmood </t>
-  </si>
-  <si>
-    <t>[{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":7,"unitPrice":13},{"code":"LT","desc":"Water Cooler (5 Gallon) ","qty":2,"unitPrice":70},{"code":"LT","desc":"Safety Shoes Italian","qty":5,"unitPrice":70},{"code":"GWH-30","desc":"Ironcap - Working At Height Helmet ","qty":1,"unitPrice":65},{"code":"HDL-001","desc":"Head lights","qty":2,"unitPrice":25},{"code":"LT","desc":"Cable Cutter 8\" ","qty":2,"unitPrice":22},{"code":"LT","desc":"Cable Cutter 10\"","qty":3,"unitPrice":25},{"code":"LT","desc":"Screw Driver (+) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Screw Driver (-) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Tie Cutter ","qty":5,"unitPrice":20},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":4,"unitPrice":20},{"code":"LT","desc":"Heat Gun","qty":1,"unitPrice":60},{"code":"LT","desc":"Silicon Gun","qty":1,"unitPrice":7},{"code":"LT","desc":"Flood Light 400 Watt","qty":1,"unitPrice":90},{"code":"ISS-100","desc":"Insulated Spanners Set (6-22)","qty":1,"unitPrice":50}]</t>
-  </si>
-  <si>
-    <t>QT-260531004</t>
-  </si>
-  <si>
-    <t>staff</t>
-  </si>
-  <si>
-    <t>Swedtel Company</t>
-  </si>
-  <si>
-    <t>Rawasy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Irfan </t>
-  </si>
-  <si>
-    <t>Technical Solution Co</t>
-  </si>
-  <si>
-    <t>BM</t>
-  </si>
-  <si>
-    <t>[{"code":"GH-60","desc":"Guardian Pro - 5D Harness","qty":1,"unitPrice":400},{"code":"GH-50","desc":"Fortress Pro - 5D Harness","qty":1,"unitPrice":350},{"code":"GDL-230","desc":"Titan Twin Static - Double Lanyard","qty":1,"unitPrice":210},{"code":"GDL-330","desc":"Titan Twin Shock- Double Lanyard","qty":1,"unitPrice":210},{"code":"GP-30","desc":"AnchorLine Adjust - Position Lanyard ","qty":1,"unitPrice":160},{"code":"GP-230","desc":"Ironhold Adjust - Position Lanyard ","qty":1,"unitPrice":160},{"code":"GSL-120","desc":"Anchorcore - Sling","qty":1,"unitPrice":30},{"code":"GCL-W100","desc":"Ironclamp - Wire Cab Lock","qty":1,"unitPrice":160},{"code":"GCL-S200","desc":"Ascendrail - Slide Cab Lock ","qty":1,"unitPrice":1000},{"code":"GSG-13","desc":"GripX - Safety Gloves","qty":1,"unitPrice":3},{"code":"GSG-21","desc":"GripX Pro - Safety Gloves","qty":1,"unitPrice":8},{"code":"ISS-100","desc":"Insulated Spanners Set (6-22)","qty":1,"unitPrice":50},{"code":"GRF-A10","desc":"Guard - Rope Fall Arrestor","qty":1,"unitPrice":300},{"code":"GRF-A20","desc":"Guard - Rope Fall Arrestor","qty":1,"unitPrice":300},{"code":"GR-P200","desc":"Anchorline - Rope 200M","qty":1,"unitPrice":700},{"code":"GWH-30","desc":"Ironcap - Working At Height Helmet ","qty":1,"unitPrice":70},{"code":"NM-001","desc":"Engineer Helmet","qty":1,"unitPrice":30},{"code":"GCR-100","desc":"Corelock - Carabiner","qty":1,"unitPrice":15},{"code":"H110","desc":"Label Machine Brother","qty":1,"unitPrice":180},{"code":"GRB-25","desc":"Rigger Bag","qty":1,"unitPrice":70},{"code":"FAK-100","desc":"First Aid Kit","qty":1,"unitPrice":65},{"code":"LT","desc":"Bosch Laser Meter 150m","qty":1,"unitPrice":1400},{"code":"LT","desc":"Multimeter (SANWA)","qty":1,"unitPrice":180},{"code":"LT","desc":"AC/DC Clamp Meter ","qty":1,"unitPrice":170},{"code":"LT","desc":"Clamp Meter (Kuoritsu)","qty":1,"unitPrice":190},{"code":"LT","desc":"Crimping Tool RJ 45","qty":1,"unitPrice":60},{"code":"LT","desc":"Power Crimper 6-50MM Size","qty":1,"unitPrice":85},{"code":"LT","desc":"RJ 45 Tester","qty":1,"unitPrice":55},{"code":"LT","desc":"Combination Wrench Set (6-32) 14 pcs Insulated","qty":1,"unitPrice":65},{"code":"LT","desc":"Combination Wrench Set (6-32) 25 pcs Insulated","qty":1,"unitPrice":115},{"code":"CMP-001","desc":"Compass","qty":1,"unitPrice":100},{"code":"CMPD-001","desc":"Digital Compass","qty":1,"unitPrice":200},{"code":"LT","desc":"Compass With Mirror ","qty":1,"unitPrice":75},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":1,"unitPrice":20},{"code":"LT","desc":"Socket Wrench Set 24 pcs 1/2\"","qty":1,"unitPrice":125},{"code":"LT","desc":"Adjustable Wrench 10\"","qty":1,"unitPrice":30},{"code":"LT","desc":"Adjustable Wrench 12\"","qty":1,"unitPrice":40},{"code":"LT","desc":"Screw Driver (+) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Screw Driver (-) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Insulated Screw Driver Set With Tester","qty":1,"unitPrice":70},{"code":"LT","desc":"Insulated Screw Driver Set With Tester China","qty":1,"unitPrice":35},{"code":"LT","desc":"Hacksaw Frame With Blade","qty":1,"unitPrice":18},{"code":"LT","desc":"Allen Key Set 1.5–10mm","qty":1,"unitPrice":60},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":1,"unitPrice":40},{"code":"LT","desc":"Electrical Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Long Nose Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Cutter Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Vice Grip Plier 10\"","qty":1,"unitPrice":35},{"code":"LT","desc":"Cable Cutter 8\" ","qty":1,"unitPrice":22},{"code":"LT","desc":"Cable Cutter 10\"","qty":1,"unitPrice":25},{"code":"LT","desc":"Tie Cutter ","qty":1,"unitPrice":20},{"code":"LT","desc":"Safety Shoes Italian","qty":1,"unitPrice":70},{"code":"LT","desc":"Electrical Gloves Class 1","qty":1,"unitPrice":85},{"code":"LT","desc":"Electrical Gloves Class 0 ","qty":1,"unitPrice":65},{"code":"LT","desc":"Zamil Aluminium Ladder 3 Step","qty":1,"unitPrice":125},{"code":"LT","desc":"Zamil Aluminium Ladder 5 Step","qty":1,"unitPrice":180},{"code":"LT","desc":"Flood Light 400 Watt","qty":1,"unitPrice":90},{"code":"LT","desc":"Heat Gun","qty":1,"unitPrice":60},{"code":"LT","desc":"Drill Machine","qty":1,"unitPrice":190},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":1,"unitPrice":13},{"code":"GBV-100-XL","desc":"ViziGuard - Safety Vest","qty":1,"unitPrice":13},{"code":"LT","desc":"Measuring Tape 10m (Dewesser Germany)","qty":1,"unitPrice":25},{"code":"HDL-001","desc":"Head lights","qty":1,"unitPrice":25},{"code":"LT","desc":"3M Eye Protection Googles ","qty":1,"unitPrice":40},{"code":"GRK-100","desc":"ResQ Pro - Rescue Kit ","qty":1,"unitPrice":1300},{"code":"LT","desc":"Measuring Tape 5m (Dewesser Germany)","qty":1,"unitPrice":15},{"code":"LT","desc":"Measuring Tape 30M","qty":1,"unitPrice":35},{"code":"LT","desc":"Measuring Tape 50M","qty":1,"unitPrice":45}]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Vision Contractring Company </t>
-  </si>
-  <si>
-    <t>QT-260531005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adil Awan </t>
+    <t>New Telecom</t>
   </si>
   <si>
     <t>[{"code":"LT","desc":"Insulated Screw Driver Set With Tester","qty":7,"unitPrice":65},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":7,"unitPrice":40},{"code":"LT","desc":"Aluminum Ladder 12 Step ","qty":7,"unitPrice":205},{"code":"LT","desc":"Ring Spanner Set HQ 6*22 PCS","qty":7,"unitPrice":60},{"code":"GSG-21","desc":"GripX Pro - Safety Gloves","qty":7,"unitPrice":6},{"code":"LT","desc":"Cable Cutter 18\"","qty":7,"unitPrice":40},{"code":"LT","desc":"Splicer Knife (STANLEY)","qty":7,"unitPrice":18},{"code":"LT","desc":"Adjustable Wrench 10\"","qty":7,"unitPrice":30},{"code":"LT","desc":"AC/DC Clamp Meter ","qty":7,"unitPrice":150},{"code":"LT","desc":"Hammer Brazil 500g","qty":7,"unitPrice":25},{"code":"H110","desc":"Brother-H110","qty":7,"unitPrice":180},{"code":"LT","desc":"Electrical Plier (Dewesser Germany)","qty":7,"unitPrice":18},{"code":"LT","desc":"Cutter Plier Red Small ","qty":7,"unitPrice":14},{"code":"LT","desc":"Long Nose Plier (Dewesser Germany)","qty":7,"unitPrice":18},{"code":"LT","desc":"Hammer Drill 13MM","qty":7,"unitPrice":130},{"code":"LT","desc":"Angel Grinder (BOSCH)","qty":7,"unitPrice":140},{"code":"LT","desc":"Socket Wrench Set 24 pcs 1/2\"","qty":7,"unitPrice":125},{"code":"LT","desc":"Measuring Tape 7.5m (Dewesser Germany)","qty":7,"unitPrice":15},{"code":"LT","desc":"Sheet Cutter (STANLEY)","qty":7,"unitPrice":40},{"code":"GWH-30","desc":"Ironcap - Working At Height Helmet ","qty":7,"unitPrice":50},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":4,"unitPrice":11},{"code":"GBV-100-XL","desc":"ViziGuard - Safety Vest","qty":3,"unitPrice":11},{"code":"LT","desc":"Spanner 10MM ","qty":7,"unitPrice":6},{"code":"LT","desc":"T Spanner 12MM  ","qty":7,"unitPrice":9},{"code":"LT","desc":"T Spanner 13MM  ","qty":7,"unitPrice":9},{"code":"LT","desc":"T Spanner 14MM  ","qty":7,"unitPrice":10},{"code":"LT","desc":"T Spanner 15MM  ","qty":7,"unitPrice":10},{"code":"LT","desc":"T Spanner 17MM  ","qty":7,"unitPrice":10},{"code":"LT","desc":"T Spanner 19MM  ","qty":7,"unitPrice":12},{"code":"LT","desc":"Hand Crimping Tool 6-50mm","qty":7,"unitPrice":85},{"code":"LT","desc":"Steel Tool Box","qty":7,"unitPrice":65}]</t>
@@ -139,72 +163,48 @@
     <t>QT-260601001</t>
   </si>
   <si>
-    <t>Smart lines</t>
-  </si>
-  <si>
     <t xml:space="preserve">Faheem </t>
   </si>
   <si>
+    <t>Shah</t>
+  </si>
+  <si>
+    <t>FTC</t>
+  </si>
+  <si>
     <t>[{"code":"LT","desc":"Digital Vernier Caliper 6\"","qty":1,"unitPrice":140},{"code":"GP-30","desc":"AnchorLine Adjust - Position Lanyard ","qty":3,"unitPrice":150},{"code":"LT","desc":"Measuring Tape 100m ","qty":1,"unitPrice":70},{"code":"GSG-21","desc":"GripX Pro - Safety Gloves","qty":4,"unitPrice":8},{"code":"LT","desc":"Safety Panaflex 60x90 CM","qty":1,"unitPrice":40}]</t>
   </si>
   <si>
-    <t>Dorr-Almas.Est</t>
-  </si>
-  <si>
     <t>QT-260601002</t>
   </si>
   <si>
-    <t>FTC</t>
-  </si>
-  <si>
     <t>Jawad Malik</t>
   </si>
   <si>
-    <t>DAEM COMPANY FOR TRADING</t>
-  </si>
-  <si>
-    <t>I-man co</t>
-  </si>
-  <si>
-    <t>Xad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Company KAREEM SWAR </t>
-  </si>
-  <si>
-    <t>Alpha Global</t>
-  </si>
-  <si>
-    <t>New Telecom</t>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Newera</t>
+  </si>
+  <si>
+    <t>ZCC</t>
+  </si>
+  <si>
+    <t>Thrones Arabia</t>
+  </si>
+  <si>
+    <t>WAJDA GLOBAL COMPANY</t>
   </si>
   <si>
     <t>[{"code":"GH-50","desc":"Fortress Pro - 5D Harness","qty":1,"unitPrice":350},{"code":"GDL-230","desc":"Titan Twin Static - Double Lanyard","qty":1,"unitPrice":210},{"code":"GP-30","desc":"AnchorLine Adjust - Position Lanyard ","qty":1,"unitPrice":160},{"code":"GSL-120","desc":"Anchorcore - Sling","qty":1,"unitPrice":30},{"code":"GSG-13","desc":"GripX - Safety Gloves","qty":1,"unitPrice":3},{"code":"GSG-21","desc":"GripX Pro - Safety Gloves","qty":1,"unitPrice":8},{"code":"GCR-100","desc":"Corelock - Carabiner","qty":1,"unitPrice":15},{"code":"GCL-W100","desc":"Ironclamp - Wire Cab Lock","qty":1,"unitPrice":160},{"code":"GCL-S200","desc":"Ascendrail - Slide Cab Lock ","qty":1,"unitPrice":1000},{"code":"GRF-A10","desc":"Guard - Rope Fall Arrestor","qty":1,"unitPrice":300},{"code":"GRF-A20","desc":"Guard - Rope Fall Arrestor","qty":1,"unitPrice":300},{"code":"GR-P200","desc":"Anchorline - Rope 200M","qty":1,"unitPrice":700},{"code":"GRB-25","desc":"Rigger Bag","qty":1,"unitPrice":70},{"code":"ISS-100","desc":"Insulated Spanners Set (6-22)","qty":1,"unitPrice":50},{"code":"H110","desc":"Label Machine (Brother)","qty":1,"unitPrice":180},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":1,"unitPrice":13},{"code":"GBV-100-XL","desc":"ViziGuard - Safety Vest","qty":1,"unitPrice":13},{"code":"LT","desc":"Safety Shoes Italian","qty":1,"unitPrice":70},{"code":"GWH-30","desc":"Ironcap - Working At Height Helmet ","qty":1,"unitPrice":70},{"code":"NM-001","desc":"Engineer Helmet","qty":1,"unitPrice":30},{"code":"FAK-100","desc":"First Aid Kit","qty":1,"unitPrice":65},{"code":"CMP-001","desc":"Compass","qty":1,"unitPrice":100},{"code":"CMPD-001","desc":"Digital Compass","qty":1,"unitPrice":200},{"code":"LT","desc":"Compass With Mirror ","qty":1,"unitPrice":75},{"code":"GRK-100","desc":"ResQ Pro - Rescue Kit ","qty":1,"unitPrice":1300},{"code":"HDL-001","desc":"Head lights","qty":1,"unitPrice":25},{"code":"LT","desc":"Bosch Laser Meter 150m","qty":1,"unitPrice":1400},{"code":"LT","desc":"Multimeter (SANWA)","qty":1,"unitPrice":180},{"code":"LT","desc":"Clamp Meter (Kuoritsu)","qty":1,"unitPrice":190},{"code":"LT","desc":"AC/DC Clamp Meter ","qty":1,"unitPrice":170},{"code":"LT","desc":"Drill Machine","qty":1,"unitPrice":190},{"code":"LT","desc":"Heat Gun","qty":1,"unitPrice":60},{"code":"LT","desc":"Screw Driver (+) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Screw Driver (-) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Insulated Screw Driver Set With Tester","qty":1,"unitPrice":70},{"code":"LT","desc":"Insulated Screw Driver Set With Tester China","qty":1,"unitPrice":35},{"code":"LT","desc":"Torx Screw Driver (Taiwan)","qty":1,"unitPrice":30},{"code":"LT","desc":"Allen Key Set 1.5–10mm","qty":1,"unitPrice":60},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":1,"unitPrice":40},{"code":"LT","desc":"Hacksaw Frame With Blade","qty":1,"unitPrice":18},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":1,"unitPrice":20},{"code":"LT","desc":"Electrical Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Long Nose Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Monkey Plier 10\"","qty":1,"unitPrice":55},{"code":"LT","desc":"Cutter Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Cable Cutter 8\" ","qty":1,"unitPrice":22},{"code":"LT","desc":"Cable Cutter 10\"","qty":1,"unitPrice":25},{"code":"LT","desc":"Cable Cutter 18\"","qty":1,"unitPrice":40},{"code":"LT","desc":"Vice Grip Plier 10\"","qty":1,"unitPrice":35},{"code":"LT","desc":"Zamil Aluminium Ladder 3 Step","qty":1,"unitPrice":125},{"code":"LT","desc":"Zamil Aluminium Ladder 5 Step","qty":1,"unitPrice":180},{"code":"LT","desc":"Aluminum Ladder 12 Step ","qty":1,"unitPrice":215},{"code":"LT","desc":"Tie Cutter ","qty":1,"unitPrice":20},{"code":"LT","desc":"Electrical Gloves Class 1","qty":1,"unitPrice":85},{"code":"LT","desc":"Electrical Gloves Class 0 ","qty":1,"unitPrice":65},{"code":"LT","desc":"Flood Light 400 Watt","qty":1,"unitPrice":90},{"code":"LT","desc":"Measuring Tape 5m (Dewesser Germany)","qty":1,"unitPrice":15},{"code":"LT","desc":"Measuring Tape 10m (Dewesser Germany)","qty":1,"unitPrice":25},{"code":"LT","desc":"Measuring Tape 30M","qty":1,"unitPrice":35},{"code":"LT","desc":"Measuring Tape 7.5m (Dewesser Germany)","qty":1,"unitPrice":15},{"code":"LT","desc":"Measuring Tape 50M","qty":1,"unitPrice":45},{"code":"LT","desc":"Measuring Tape 100m ","qty":1,"unitPrice":70},{"code":"LT","desc":"Socket Wrench Set 24 pcs 1/2\"","qty":1,"unitPrice":125},{"code":"LT","desc":"Combination Wrench Set (6-32) 14 pcs Insulated","qty":1,"unitPrice":65},{"code":"LT","desc":"Combination Wrench Set (6-32) 25 pcs Insulated","qty":1,"unitPrice":115},{"code":"LT","desc":"Adjustable Wrench 10\"","qty":1,"unitPrice":30},{"code":"LT","desc":"Adjustable Wrench 12\"","qty":1,"unitPrice":40},{"code":"LT","desc":"Power Crimper 6-50MM Size","qty":1,"unitPrice":85},{"code":"LT","desc":"Crimping Tool RJ 45","qty":1,"unitPrice":60},{"code":"LT","desc":"RJ 45 Tester","qty":1,"unitPrice":55},{"code":"LT","desc":"3M Eye Protection Googles ","qty":1,"unitPrice":40},{"code":"LT","desc":"Safety Goggels ","qty":1,"unitPrice":5},{"code":"LT","desc":"Powder Fire Extinguisher 2 kg With 6 Months Sticker","qty":1,"unitPrice":50},{"code":"LT","desc":"Powder Fire Extinguisher 3 kg With 6 Months Sticker","qty":1,"unitPrice":55}]</t>
   </si>
   <si>
-    <t>Shah</t>
-  </si>
-  <si>
     <t>QT-260601003</t>
   </si>
   <si>
     <t>M.Abbas</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Newera</t>
-  </si>
-  <si>
-    <t>ZCC</t>
-  </si>
-  <si>
-    <t>Thrones Arabia</t>
-  </si>
-  <si>
-    <t>WAJDA GLOBAL COMPANY</t>
-  </si>
-  <si>
     <t>[{"code":"GH-60","desc":"Guardian Pro - 5D Harness","qty":1,"unitPrice":380},{"code":"GH-50","desc":"Fortress Pro - 5D Harness","qty":1,"unitPrice":315},{"code":"GDL-230","desc":"Titan Twin Static - Double Lanyard","qty":1,"unitPrice":200},{"code":"GP-30","desc":"AnchorLine Adjust - Position Lanyard ","qty":1,"unitPrice":150},{"code":"GSL-120","desc":"Anchorcore - Sling","qty":1,"unitPrice":30},{"code":"GCR-100","desc":"Corelock - Carabiner","qty":1,"unitPrice":15},{"code":"GCL-W100","desc":"Ironclamp - Wire Cab Lock","qty":1,"unitPrice":150},{"code":"GCL-S200","desc":"Ascendrail - Slide Cab Lock ","qty":1,"unitPrice":1000},{"code":"GRF-A10","desc":"Guard - Rope Fall Arrestor","qty":1,"unitPrice":300},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":1,"unitPrice":13},{"code":"GBV-100-XL","desc":"ViziGuard - Safety Vest","qty":1,"unitPrice":13},{"code":"GSG-13","desc":"GripX - Safety Gloves","qty":1,"unitPrice":3},{"code":"GSG-21","desc":"GripX Pro - Safety Gloves","qty":1,"unitPrice":8},{"code":"LT","desc":"Safety Shoes Italian","qty":1,"unitPrice":70},{"code":"ISS-100","desc":"Insulated Spanners Set (6-22)","qty":1,"unitPrice":50},{"code":"H110","desc":"Label Machine (Brother)","qty":1,"unitPrice":180},{"code":"HDL-001","desc":"Head lights","qty":1,"unitPrice":25},{"code":"CMP-001","desc":"Compass","qty":1,"unitPrice":100},{"code":"CMPD-001","desc":"Digital Compass","qty":1,"unitPrice":200},{"code":"LT","desc":"Compass With Mirror ","qty":1,"unitPrice":75},{"code":"GRB-25","desc":"Rigger Bag","qty":1,"unitPrice":70},{"code":"GWH-30","desc":"Ironcap - Working At Height Helmet ","qty":1,"unitPrice":60},{"code":"NM-001","desc":"Engineer Helmet","qty":1,"unitPrice":30},{"code":"FAK-100","desc":"First Aid Kit","qty":1,"unitPrice":60},{"code":"GRK-100","desc":"ResQ Pro - Rescue Kit ","qty":1,"unitPrice":1350},{"code":"LT","desc":"Bosch Laser Meter 150m","qty":1,"unitPrice":1325},{"code":"LT","desc":"Drill Machine","qty":1,"unitPrice":190},{"code":"LT","desc":"Heat Gun","qty":1,"unitPrice":60},{"code":"LT","desc":"Screw Driver (+) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Screw Driver (-) Big (Taiwan)","qty":1,"unitPrice":12},{"code":"LT","desc":"Combination Wrench Set (6-32) 14 pcs Insulated","qty":1,"unitPrice":65},{"code":"LT","desc":"Combination Wrench Set (6-32) 25 pcs Insulated","qty":1,"unitPrice":115},{"code":"LT","desc":"Socket Wrench Set 24 pcs 1/2\"","qty":1,"unitPrice":125},{"code":"LT","desc":"Adjustable Wrench 10\"","qty":1,"unitPrice":30},{"code":"LT","desc":"Adjustable Wrench 12\"","qty":1,"unitPrice":40},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":1,"unitPrice":20},{"code":"LT","desc":"Hacksaw Frame With Blade","qty":1,"unitPrice":18},{"code":"LT","desc":"Allen Key Set 1.5–10mm","qty":1,"unitPrice":60},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":1,"unitPrice":40},{"code":"LT","desc":"Electrical Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Electrical Gloves Class 1","qty":1,"unitPrice":85},{"code":"LT","desc":"Electrical Gloves Class 0 ","qty":1,"unitPrice":65},{"code":"LT","desc":"Long Nose Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Monkey Plier 10\"","qty":1,"unitPrice":55},{"code":"LT","desc":"Cable Drum 50M Germany","qty":1,"unitPrice":125},{"code":"LT","desc":"Cable Cutter 8\" ","qty":1,"unitPrice":22},{"code":"LT","desc":"Cable Cutter 10\"","qty":1,"unitPrice":25},{"code":"LT","desc":"Cable Cutter 18\"","qty":1,"unitPrice":40},{"code":"LT","desc":"Tie Cutter ","qty":1,"unitPrice":20},{"code":"LT","desc":"Vice Grip Plier 10\"","qty":1,"unitPrice":35},{"code":"LT","desc":"Zamil Aluminium Ladder 3 Step","qty":1,"unitPrice":125},{"code":"LT","desc":"Zamil Aluminium Ladder 5 Step","qty":1,"unitPrice":180},{"code":"LT","desc":"Aluminum Ladder 12 Step ","qty":1,"unitPrice":215},{"code":"LT","desc":"Flood Light 400 Watt","qty":1,"unitPrice":90},{"code":"LT","desc":"Measuring Tape 5m (Dewesser Germany)","qty":1,"unitPrice":15},{"code":"LT","desc":"Measuring Tape 10m (Dewesser Germany)","qty":1,"unitPrice":25},{"code":"LT","desc":"Measuring Tape 7.5m (Dewesser Germany)","qty":1,"unitPrice":15},{"code":"LT","desc":"Measuring Tape 30M","qty":1,"unitPrice":35},{"code":"LT","desc":"Measuring Tape 50M","qty":1,"unitPrice":45},{"code":"LT","desc":"Measuring Tape 100m ","qty":1,"unitPrice":70},{"code":"LT","desc":"Powder Fire Extinguisher 2 kg With 6 Months Sticker","qty":1,"unitPrice":50},{"code":"LT","desc":"Powder Fire Extinguisher 3 kg With 6 Months Sticker","qty":1,"unitPrice":55},{"code":"LT","desc":"Hand Crimping Tool 6-50mm","qty":1,"unitPrice":85},{"code":"LT","desc":"Crimping Tool RJ 45","qty":1,"unitPrice":60},{"code":"LT","desc":"RJ 45 Tester","qty":1,"unitPrice":55},{"code":"LT","desc":"Insulated Screw Driver Set With Tester China","qty":1,"unitPrice":35}]</t>
   </si>
   <si>
@@ -613,7 +613,7 @@
     <t>QT-260629054</t>
   </si>
   <si>
-    <t>[{"code":"LT","desc":"Garmin GPS ","qty":1,"unitPrice":750},{"code":"LT","desc":"Bosch Laser Meter 150m","qty":1,"unitPrice":1400},{"code":"LT","desc":"Elcometer","qty":1,"unitPrice":350}]</t>
+    <t>[{"code":"LT","desc":"Garmin GPS ","qty":5,"unitPrice":750},{"code":"LT","desc":"Elcometer","qty":5,"unitPrice":350}]</t>
   </si>
   <si>
     <t>QT-260630055</t>
@@ -658,7 +658,7 @@
     <t>QT-260703006</t>
   </si>
   <si>
-    <t>[{"code":"HDL-001","desc":"Head lights","qty":6,"unitPrice":25},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":3,"unitPrice":13},{"code":"GBV-100-XL","desc":"ViziGuard - Safety Vest","qty":6,"unitPrice":13},{"code":"NM-001","desc":"Engineer Helmet","qty":3,"unitPrice":30},{"code":"GWH-50","desc":"Ironcap Pro - Working At Height Helmet ","qty":3,"unitPrice":65},{"code":"LT","desc":"Safety Shoes Italian","qty":5,"unitPrice":70},{"code":"GDL-230","desc":"Titan Twin Static - Double Lanyard","qty":9,"unitPrice":185},{"code":"GH-50","desc":"Fortress Pro - 5D Harness","qty":5,"unitPrice":315},{"code":"GP-30","desc":"AnchorLine Adjust - Position Lanyard ","qty":5,"unitPrice":150},{"code":"LT","desc":"Flood Light 400 Watt","qty":1,"unitPrice":90},{"code":"GRB-25","desc":"Rigger Bag","qty":3,"unitPrice":70},{"code":"GR-P200","desc":"Anchorline - Rope 200M","qty":2,"unitPrice":690},{"code":"GSP-200","desc":"Reely - Single Pulley","qty":1,"unitPrice":150},{"code":"LT","desc":"Cable Cutter 18\"","qty":1,"unitPrice":40},{"code":"LT","desc":"Tie Cutter Big","qty":1,"unitPrice":20},{"code":"LT","desc":"Steel Tool Box","qty":2,"unitPrice":65},{"code":"LT","desc":"Hand Crimping Tool 6-50mm","qty":1,"unitPrice":85}]</t>
+    <t>[{"code":"GR-P200","desc":"Anchorline - Rope 200M","qty":3,"unitPrice":690},{"code":"GH-50","desc":"Fortress Pro - 5D Harness","qty":3,"unitPrice":315},{"code":"GP-30","desc":"AnchorLine Adjust - Position Lanyard ","qty":3,"unitPrice":150},{"code":"GDL-230","desc":"Titan Twin Static - Double Lanyard","qty":3,"unitPrice":185},{"code":"LT","desc":"Safety Shoes Italian","qty":1,"unitPrice":70},{"code":"NM-001","desc":"Engineer Helmet","qty":1,"unitPrice":30},{"code":"LT","desc":"Steel Tool Box","qty":1,"unitPrice":65},{"code":"LT","desc":"Silicon Box","qty":1,"unitPrice":95},{"code":"GWH-50","desc":"Ironcap Pro - Working At Height Helmet ","qty":2,"unitPrice":65},{"code":"GBV-100-L","desc":"ViziGuard - Safety Vest","qty":3,"unitPrice":13}]</t>
   </si>
   <si>
     <t>QT-260703007</t>
@@ -820,7 +820,7 @@
     <t>QT-260719024</t>
   </si>
   <si>
-    <t>[{"code":"LT","desc":"Safety Shoes Italian","qty":12,"unitPrice":80},{"code":"GBV-100-XL","desc":"ViziGuard - Safety Vest","qty":24,"unitPrice":13},{"code":"GWH-50","desc":"Ironcap Pro - Working At Height Helmet ","qty":21,"unitPrice":65},{"code":"HDL-001","desc":"Head lights","qty":6,"unitPrice":30},{"code":"LT","desc":"Powder Fire Extinguisher 3 kg With 6 Months Sticker","qty":2,"unitPrice":60},{"code":"FAK-100","desc":"First Aid Kit","qty":4,"unitPrice":65},{"code":"GSG-13","desc":"GripX - Safety Gloves","qty":44,"unitPrice":4},{"code":"GH-50","desc":"Fortress Pro - 5D Harness","qty":4,"unitPrice":350},{"code":"GDL-330","desc":"Titan Twin Shock- Double Lanyard","qty":12,"unitPrice":250},{"code":"GP-30","desc":"AnchorLine Adjust - Position Lanyard ","qty":6,"unitPrice":200},{"code":"GRB-25","desc":"Rigger Bag","qty":16,"unitPrice":80},{"code":"LT","desc":"Steel Tool Box","qty":3,"unitPrice":70},{"code":"GR-P100","desc":"Anchorline - Rope 100M","qty":3,"unitPrice":600},{"code":"GR-P200","desc":"Anchorline - Rope 200M","qty":4,"unitPrice":1000},{"code":"GSL-120","desc":"Anchorcore - Sling","qty":3,"unitPrice":40},{"code":"GDP-200","desc":"Twiny - Double Pulley","qty":6,"unitPrice":200},{"code":"GCR-100","desc":"Corelock - Carabiner","qty":1,"unitPrice":15},{"code":"LT","desc":"Flood Light 400 Watt","qty":4,"unitPrice":100}]</t>
+    <t>[{"code":"LT","desc":"Safety Shoes Italian","qty":12,"unitPrice":80},{"code":"GBV-100-XL","desc":"ViziGuard - Safety Vest","qty":24,"unitPrice":13},{"code":"GWH-50","desc":"Ironcap Pro - Working At Height Helmet ","qty":21,"unitPrice":65},{"code":"HDL-001","desc":"Head lights","qty":6,"unitPrice":30},{"code":"LT","desc":"Powder Fire Extinguisher 3 kg With 6 Months Sticker","qty":2,"unitPrice":60},{"code":"FAK-100","desc":"First Aid Kit","qty":4,"unitPrice":65},{"code":"GSG-13","desc":"GripX - Safety Gloves","qty":44,"unitPrice":4},{"code":"GH-50","desc":"Fortress Pro - 5D Harness","qty":4,"unitPrice":350},{"code":"GDL-230","desc":"Titan Twin Static - Double Lanyard","qty":12,"unitPrice":210},{"code":"GP-30","desc":"AnchorLine Adjust - Position Lanyard ","qty":6,"unitPrice":200},{"code":"GRB-25","desc":"Rigger Bag","qty":16,"unitPrice":80},{"code":"LT","desc":"Steel Tool Box","qty":3,"unitPrice":70},{"code":"GR-P100","desc":"Anchorline - Rope 100M","qty":3,"unitPrice":600},{"code":"GR-P200","desc":"Anchorline - Rope 200M","qty":4,"unitPrice":1000},{"code":"GSL-120","desc":"Anchorcore - Sling","qty":3,"unitPrice":40},{"code":"GDP-200","desc":"Twiny - Double Pulley","qty":6,"unitPrice":200},{"code":"GCR-100","desc":"Corelock - Carabiner","qty":1,"unitPrice":15},{"code":"LT","desc":"Flood Light 400 Watt","qty":4,"unitPrice":100}]</t>
   </si>
   <si>
     <t>QT-260719025</t>
@@ -848,6 +848,30 @@
   </si>
   <si>
     <t>[{"code":"LT","desc":"Electrical Gloves Class 0 ","qty":1,"unitPrice":65},{"code":"GSG-13","desc":"GripX - Safety Gloves","qty":4,"unitPrice":3},{"code":"LT","desc":"Safety Shoes Italian","qty":1,"unitPrice":70},{"code":"HDL-001","desc":"Head lights","qty":3,"unitPrice":20},{"code":"FAK-100","desc":"First Aid Kit","qty":1,"unitPrice":50},{"code":"LT","desc":"Powder Fire Extinguisher 4 kg With 6 Months Sticker","qty":1,"unitPrice":45},{"code":"GRF-A20","desc":"Guard - Rope Fall Arrestor","qty":1,"unitPrice":250},{"code":"LT","desc":"Multimeter (SANWA)","qty":2,"unitPrice":180},{"code":"LT","desc":"AC/DC Clamp Meter ","qty":1,"unitPrice":150},{"code":"LT","desc":"Bosch Laser Meter 150m","qty":1,"unitPrice":1350},{"code":"H110","desc":"Brother-H110","qty":1,"unitPrice":180},{"code":"CMPD-001","desc":"Digital Compass","qty":1,"unitPrice":160},{"code":"LT","desc":"Measuring Tape 5m (Dewesser Germany)","qty":1,"unitPrice":15},{"code":"LT","desc":"Water Level Deweser Germany 40cm ","qty":1,"unitPrice":22},{"code":"LT","desc":"Hacksaw Frame With Blade","qty":1,"unitPrice":15},{"code":"LT","desc":"Claw Hammer","qty":1,"unitPrice":18},{"code":"LT","desc":"Steel Tool Box","qty":1,"unitPrice":65},{"code":"LT","desc":"Combination Spanner 8MM","qty":1,"unitPrice":8},{"code":"LT","desc":"Combination Spanner 10MM","qty":1,"unitPrice":8},{"code":"LT","desc":"Combination Spanner 11MM","qty":1,"unitPrice":8},{"code":"LT","desc":"Combination Spanner 12MM","qty":1,"unitPrice":10},{"code":"LT","desc":"Combination Spanner 13MM","qty":3,"unitPrice":8},{"code":"LT","desc":"Combination Spanner 14MM","qty":1,"unitPrice":9},{"code":"LT","desc":"Combination Spanner 15MM","qty":1,"unitPrice":9},{"code":"LT","desc":"Combination Spanner 16MM","qty":2,"unitPrice":9.5},{"code":"LT","desc":"Combination Spanner 17MM","qty":2,"unitPrice":10},{"code":"LT","desc":"Combination Spanner 18MM","qty":1,"unitPrice":11},{"code":"LT","desc":"Combination Spanner 19MM","qty":1,"unitPrice":11},{"code":"LT","desc":"Combination Spanner 20MM","qty":1,"unitPrice":13},{"code":"LT","desc":"Combination Spanner 22MM","qty":1,"unitPrice":13},{"code":"LT","desc":"Combination Spanner 24MM","qty":1,"unitPrice":16},{"code":"LT","desc":"Combination Spanner 27MM","qty":1,"unitPrice":22},{"code":"LT","desc":"Combination Spanner 32MM","qty":1,"unitPrice":26},{"code":"LT","desc":"Electrical Plier (Dewesser Germany)","qty":2,"unitPrice":15},{"code":"LT","desc":"Long Nose Plier (Dewesser Germany)","qty":1,"unitPrice":15},{"code":"LT","desc":"Crimping Tool RJ 45","qty":1,"unitPrice":60},{"code":"LT","desc":"Tie Cutter Small","qty":3,"unitPrice":15},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":3,"unitPrice":18},{"code":"LT","desc":"Drill Machine","qty":1,"unitPrice":190},{"code":"LT","desc":"Cable Cutter 8\" ","qty":1,"unitPrice":22},{"code":"LT","desc":"Cable Cutter 10\"","qty":1,"unitPrice":25},{"code":"LT","desc":"Flood Light 400 Watt","qty":1,"unitPrice":90},{"code":"LT","desc":"Cable Drum 50M Germany","qty":1,"unitPrice":120},{"code":"GSP-200","desc":"Reely - Single Pulley","qty":1,"unitPrice":130},{"code":"GDP-300","desc":"Twiny - Double Pulley","qty":1,"unitPrice":135},{"code":"LT","desc":"Rope 200M Local ","qty":1,"unitPrice":500},{"code":"GCR-100","desc":"Corelock - Carabiner","qty":1,"unitPrice":12},{"code":"GSL-120","desc":"Anchorcore - Sling","qty":2,"unitPrice":20},{"code":"GRB-25","desc":"Rigger Bag","qty":2,"unitPrice":60},{"code":"LT","desc":"Heat Gun Ingco ","qty":1,"unitPrice":85},{"code":"LT","desc":"Silicon Gun","qty":1,"unitPrice":7},{"code":"LT","desc":"Insulated Screw Driver Set With Tester","qty":1,"unitPrice":65},{"code":"LT","desc":"Socket Wrench Set 24 pcs 1/2\"","qty":1,"unitPrice":120},{"code":"ISS-100","desc":"Insulated Spanners Set (6-22)","qty":1,"unitPrice":40},{"code":"LT","desc":"Torx Screw Driver (Taiwan)","qty":1,"unitPrice":30},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":1,"unitPrice":40},{"code":"LT","desc":"Allen Key Set Medium Tower Star (*)","qty":1,"unitPrice":40}]</t>
+  </si>
+  <si>
+    <t>QT-260722029</t>
+  </si>
+  <si>
+    <t>Tahseen</t>
+  </si>
+  <si>
+    <t>[{"code":"GH-60","desc":"Guardian Pro - 5D Harness","qty":2,"unitPrice":380},{"code":"GP-230","desc":"Ironhold Adjust - Position Lanyard","qty":2,"unitPrice":150},{"code":"GDL-230","desc":"Titan Twin Static - Double Lanyard","qty":2,"unitPrice":200}]</t>
+  </si>
+  <si>
+    <t>QT-260728030</t>
+  </si>
+  <si>
+    <t>[{"code":"LT","desc":"Electrical Plier (Dewesser Germany)","qty":1,"unitPrice":18},{"code":"LT","desc":"Torx Screw Driver (Taiwan)","qty":1,"unitPrice":30},{"code":"LT","desc":"Allen Key Set Medium Tower","qty":1,"unitPrice":40},{"code":"LT","desc":"Cable Cutter 10\"","qty":1,"unitPrice":25},{"code":"LT","desc":"Hand Crimping Tool 6-50mm","qty":1,"unitPrice":85},{"code":"LT","desc":"Hacksaw Frame With Blade","qty":1,"unitPrice":18},{"code":"LT","desc":"Fiberglass Measuring Tape 50M","qty":1,"unitPrice":45},{"code":"LT","desc":"Splicer Knife (STANLEY USA)","qty":1,"unitPrice":20},{"code":"LT","desc":"Claw Hammer","qty":1,"unitPrice":20},{"code":"LT","desc":"Combination Spanner 13MM","qty":1,"unitPrice":8},{"code":"LT","desc":"Shovel (Steel Handle )","qty":1,"unitPrice":25},{"code":"LT","desc":"Pickaxe (wood handle)","qty":1,"unitPrice":35},{"code":"LT","desc":"Drill Machine Hilti","qty":1,"unitPrice":190}]</t>
+  </si>
+  <si>
+    <t>QT-260729031</t>
+  </si>
+  <si>
+    <t>Muhammad Tufail</t>
+  </si>
+  <si>
+    <t>[{"code":"CMPD-001","desc":"Digital Compass","qty":1,"unitPrice":200},{"code":"GDP-300","desc":"Twiny - Double Pulley","qty":1,"unitPrice":175}]</t>
   </si>
 </sst>
 </file>
@@ -1113,17 +1137,17 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.140625" customWidth="1"/>
     <col min="3" max="3" width="8.85546875" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
     <col min="7" max="7" width="7.140625" customWidth="1"/>
-    <col min="8" max="8" width="4" customWidth="1"/>
+    <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="541.7109375" customWidth="1"/>
   </cols>
@@ -1133,31 +1157,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -1165,16 +1189,16 @@
         <v>46165</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F2" s="1">
         <v>502409110</v>
@@ -1189,7 +1213,7 @@
         <v>678.5</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -1197,16 +1221,16 @@
         <v>46168</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F3" s="1">
         <v>502409110</v>
@@ -1229,13 +1253,13 @@
         <v>46170</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>24</v>
@@ -1261,16 +1285,16 @@
         <v>46171</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F5" s="1">
         <v>509079202</v>
@@ -1293,16 +1317,16 @@
         <v>46169</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F6" s="1">
         <v>539184795</v>
@@ -1317,7 +1341,7 @@
         <v>12847.8</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -1325,16 +1349,16 @@
         <v>46171</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F7" s="1">
         <v>535647223</v>
@@ -1349,7 +1373,7 @@
         <v>841.8</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -1357,16 +1381,16 @@
         <v>46172</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="F8" s="1">
         <v>537583732</v>
@@ -1381,7 +1405,7 @@
         <v>11413.75</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -1389,16 +1413,16 @@
         <v>46173</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F9" s="1">
         <v>538980173</v>
@@ -1424,7 +1448,7 @@
         <v>62</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>63</v>
@@ -1456,10 +1480,10 @@
         <v>66</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>67</v>
@@ -1488,13 +1512,13 @@
         <v>69</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F12" s="1">
         <v>502409110</v>
@@ -1520,10 +1544,10 @@
         <v>71</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>72</v>
@@ -1552,10 +1576,10 @@
         <v>74</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>75</v>
@@ -1584,10 +1608,10 @@
         <v>77</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>78</v>
@@ -1616,13 +1640,13 @@
         <v>80</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F16" s="1">
         <v>502409110</v>
@@ -1648,13 +1672,13 @@
         <v>82</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F17" s="1">
         <v>502409110</v>
@@ -1680,13 +1704,13 @@
         <v>84</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F18" s="1">
         <v>502409110</v>
@@ -1712,16 +1736,16 @@
         <v>86</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G19" s="1">
         <v>580</v>
@@ -1744,10 +1768,10 @@
         <v>88</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>89</v>
@@ -1776,10 +1800,10 @@
         <v>91</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>92</v>
@@ -1808,10 +1832,10 @@
         <v>94</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>95</v>
@@ -1840,10 +1864,10 @@
         <v>97</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>98</v>
@@ -1872,13 +1896,13 @@
         <v>100</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F24" s="1">
         <v>502409110</v>
@@ -1904,13 +1928,13 @@
         <v>102</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F25" s="1">
         <v>502409110</v>
@@ -1936,10 +1960,10 @@
         <v>104</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>105</v>
@@ -1965,7 +1989,7 @@
         <v>107</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>108</v>
@@ -1997,10 +2021,10 @@
         <v>111</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>112</v>
@@ -2029,10 +2053,10 @@
         <v>114</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>98</v>
@@ -2061,16 +2085,16 @@
         <v>116</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>117</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G30" s="1">
         <v>4700</v>
@@ -2093,10 +2117,10 @@
         <v>119</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>112</v>
@@ -2125,10 +2149,10 @@
         <v>121</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>24</v>
@@ -2157,10 +2181,10 @@
         <v>123</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>124</v>
@@ -2189,10 +2213,10 @@
         <v>126</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>127</v>
@@ -2221,10 +2245,10 @@
         <v>129</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>127</v>
@@ -2253,13 +2277,13 @@
         <v>131</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F36" s="1">
         <v>502409110</v>
@@ -2285,10 +2309,10 @@
         <v>133</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>124</v>
@@ -2317,16 +2341,16 @@
         <v>135</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>136</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G38" s="1">
         <v>17414</v>
@@ -2349,10 +2373,10 @@
         <v>138</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>139</v>
@@ -2381,10 +2405,10 @@
         <v>141</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>139</v>
@@ -2413,7 +2437,7 @@
         <v>143</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>144</v>
@@ -2445,7 +2469,7 @@
         <v>147</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>148</v>
@@ -2477,10 +2501,10 @@
         <v>151</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>152</v>
@@ -2509,10 +2533,10 @@
         <v>154</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>152</v>
@@ -2541,7 +2565,7 @@
         <v>156</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>157</v>
@@ -2573,13 +2597,13 @@
         <v>160</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="F46" s="1">
         <v>537583732</v>
@@ -2605,16 +2629,16 @@
         <v>162</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G47" s="1">
         <v>20800</v>
@@ -2637,10 +2661,10 @@
         <v>164</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>165</v>
@@ -2669,10 +2693,10 @@
         <v>167</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>112</v>
@@ -2701,13 +2725,13 @@
         <v>169</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F50" s="1">
         <v>502409110</v>
@@ -2733,7 +2757,7 @@
         <v>171</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>172</v>
@@ -2765,10 +2789,10 @@
         <v>175</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>176</v>
@@ -2797,13 +2821,13 @@
         <v>178</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F53" s="1">
         <v>502409110</v>
@@ -2829,10 +2853,10 @@
         <v>180</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>75</v>
@@ -2861,7 +2885,7 @@
         <v>182</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G55" s="1">
         <v>0</v>
@@ -2884,10 +2908,10 @@
         <v>184</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>185</v>
@@ -2916,10 +2940,10 @@
         <v>187</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>188</v>
@@ -2948,10 +2972,10 @@
         <v>190</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>191</v>
@@ -2980,10 +3004,10 @@
         <v>193</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>194</v>
@@ -3012,25 +3036,25 @@
         <v>196</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="F60" s="1">
         <v>537583732</v>
       </c>
       <c r="G60" s="1">
-        <v>2500</v>
+        <v>5500</v>
       </c>
       <c r="H60" s="1">
-        <v>375</v>
+        <v>825</v>
       </c>
       <c r="I60" s="1">
-        <v>2875</v>
+        <v>6325</v>
       </c>
       <c r="J60" s="1" t="s">
         <v>197</v>
@@ -3044,16 +3068,16 @@
         <v>198</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G61" s="1">
         <v>11962</v>
@@ -3076,10 +3100,10 @@
         <v>200</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>24</v>
@@ -3108,10 +3132,10 @@
         <v>202</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>203</v>
@@ -3140,13 +3164,13 @@
         <v>205</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F64" s="1">
         <v>502409110</v>
@@ -3172,10 +3196,10 @@
         <v>207</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>203</v>
@@ -3204,13 +3228,13 @@
         <v>209</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F66" s="1">
         <v>502409110</v>
@@ -3236,25 +3260,25 @@
         <v>211</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F67" s="1">
         <v>502409110</v>
       </c>
       <c r="G67" s="1">
-        <v>6997</v>
+        <v>4449</v>
       </c>
       <c r="H67" s="1">
-        <v>1049.55</v>
+        <v>667.35</v>
       </c>
       <c r="I67" s="1">
-        <v>8046.55</v>
+        <v>5116.3500000000004</v>
       </c>
       <c r="J67" s="1" t="s">
         <v>212</v>
@@ -3268,13 +3292,13 @@
         <v>213</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F68" s="1">
         <v>502409110</v>
@@ -3300,10 +3324,10 @@
         <v>215</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>216</v>
@@ -3332,7 +3356,7 @@
         <v>218</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D70" s="1" t="s">
         <v>219</v>
@@ -3364,13 +3388,13 @@
         <v>223</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F71" s="1">
         <v>539184795</v>
@@ -3396,7 +3420,7 @@
         <v>225</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D72" s="1" t="s">
         <v>226</v>
@@ -3428,7 +3452,7 @@
         <v>229</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D73" s="1" t="s">
         <v>226</v>
@@ -3460,7 +3484,7 @@
         <v>231</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>232</v>
@@ -3492,7 +3516,7 @@
         <v>235</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>236</v>
@@ -3524,7 +3548,7 @@
         <v>239</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>240</v>
@@ -3556,10 +3580,10 @@
         <v>243</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>194</v>
@@ -3588,10 +3612,10 @@
         <v>245</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>246</v>
@@ -3620,7 +3644,7 @@
         <v>248</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D79" s="1" t="s">
         <v>249</v>
@@ -3652,13 +3676,13 @@
         <v>252</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F80" s="1">
         <v>502409110</v>
@@ -3684,10 +3708,10 @@
         <v>254</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E81" s="1" t="s">
         <v>255</v>
@@ -3716,10 +3740,10 @@
         <v>257</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>258</v>
@@ -3748,10 +3772,10 @@
         <v>260</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E83" s="1" t="s">
         <v>136</v>
@@ -3780,10 +3804,10 @@
         <v>262</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E84" s="1" t="s">
         <v>263</v>
@@ -3812,25 +3836,25 @@
         <v>265</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G85" s="1">
-        <v>17998</v>
+        <v>17518</v>
       </c>
       <c r="H85" s="1">
-        <v>2699.7</v>
+        <v>2627.7</v>
       </c>
       <c r="I85" s="1">
-        <v>20697.7</v>
+        <v>20145.7</v>
       </c>
       <c r="J85" s="1" t="s">
         <v>266</v>
@@ -3844,13 +3868,13 @@
         <v>267</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F86" s="1">
         <v>502409110</v>
@@ -3876,10 +3900,10 @@
         <v>269</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E87" s="1" t="s">
         <v>255</v>
@@ -3908,10 +3932,10 @@
         <v>271</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>272</v>
@@ -3940,10 +3964,10 @@
         <v>274</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E89" s="1" t="s">
         <v>136</v>
@@ -3962,6 +3986,102 @@
       </c>
       <c r="J89" s="1" t="s">
         <v>275</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A90" s="2">
+        <v>46229</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="F90" s="1">
+        <v>556770056</v>
+      </c>
+      <c r="G90" s="1">
+        <v>1460</v>
+      </c>
+      <c r="H90" s="1">
+        <v>219</v>
+      </c>
+      <c r="I90" s="1">
+        <v>1679</v>
+      </c>
+      <c r="J90" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A91" s="2">
+        <v>46231</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G91" s="1">
+        <v>559</v>
+      </c>
+      <c r="H91" s="1">
+        <v>83.85</v>
+      </c>
+      <c r="I91" s="1">
+        <v>642.85</v>
+      </c>
+      <c r="J91" s="1" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A92" s="2">
+        <v>46232</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="F92" s="1">
+        <v>547278259</v>
+      </c>
+      <c r="G92" s="1">
+        <v>375</v>
+      </c>
+      <c r="H92" s="1">
+        <v>56.25</v>
+      </c>
+      <c r="I92" s="1">
+        <v>431.25</v>
+      </c>
+      <c r="J92" s="1" t="s">
+        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>